<commit_message>
Finalizando - Santander- Excel com IA e Claude DIO
</commit_message>
<xml_diff>
--- a/Cursos/Santander- Excel com IA e Claude/Criando Um Organizador de Declaração de Imposto de Renda/Controle_IR_Declaracao.xlsx
+++ b/Cursos/Santander- Excel com IA e Claude/Criando Um Organizador de Declaração de Imposto de Renda/Controle_IR_Declaracao.xlsx
@@ -1866,7 +1866,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:F30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2113,8 +2113,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2126,7 +2126,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:F32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2401,8 +2401,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2414,7 +2414,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF1F4E78"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:D24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2645,8 +2645,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2658,7 +2658,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF1F4E78"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B2:C26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2832,8 +2832,8 @@
     <hyperlink ref="B15" r:id="rId10" location="Resumo!A1" display="📊  Resumo e Status"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2845,7 +2845,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:D19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3014,8 +3014,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3027,7 +3027,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:F18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3193,8 +3193,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3206,7 +3206,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:G30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3488,8 +3488,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3501,7 +3501,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:F30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3749,8 +3749,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3762,7 +3762,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:G30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -4044,8 +4044,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4057,7 +4057,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:F35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -4348,8 +4348,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4361,7 +4361,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:F25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -4577,8 +4577,8 @@
     <hyperlink ref="B2" r:id="rId1" location="Menu!A1" display="◀  Voltar ao Menu"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>